<commit_message>
Clean up redundant files, update build script, and add client marketing/case studies requirements
</commit_message>
<xml_diff>
--- a/STEAMEE_Client_Dashboard_Spec.xlsx
+++ b/STEAMEE_Client_Dashboard_Spec.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1. Overview Hub" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2. User Analytics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3. Store Operations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4. Rider Logistics" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5. Finance &amp; Revenue" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6. Growth &amp; Marketing" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="7. Complaint &amp; Quality" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="8. TAT Analytics" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="9. Ironer &amp; Staff Performance" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="10. Masters Configuration" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="11. Operational Lists &amp; Tables" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Overview Hub" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. User Analytics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Store Operations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Rider Logistics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Finance &amp; Revenue" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Growth &amp; Marketing" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Complaint &amp; Quality" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. TAT Analytics" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Ironer &amp; Staff Performance" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Masters Configuration" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. Operational Lists &amp; Tables" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. Portal + MoEngage (Mktg)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13. Metabase + MoEngage (Mktg)" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,8 +77,14 @@
       <color rgb="00A05A00"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00856404"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +136,11 @@
         <fgColor rgb="00FFEFA6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -155,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -185,6 +198,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -554,7 +576,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -1389,7 +1411,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -2224,7 +2246,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -3181,6 +3203,2052 @@
       <c r="I21" s="4" t="inlineStr">
         <is>
           <t>Ready to Build</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001B365D"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STEAMEE — Portal + MoEngage (Marketing Architecture)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard Element Type</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Element Name / Attributes</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>What it Shows (Plain English)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Target Portal Role / User</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Suggested Visualization</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Business Purpose &amp; Decision Impact</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Available Filters</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Source KPI Map</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Build Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Acquisition (P0)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>[D01] User Acquisition</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>New customers; New customer orders; AOV (first order); First-order item mix; Spend-to-new ratio (if spend joined)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Trend line of new customers; stacked bar by source; map/table by city &amp; store; item-mix bar; first-order AOV KPI</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>See where new customers come from and what they buy on first order, so we can judge which sources/cities/stores produce quality acquisition.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Acquisition Source; Order Channel; City; Store; Garment/Item Category. Granularity: Daily / Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Conversion (P0)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[D02] User Conversion Funnel</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Visitors; Signups; Profiles created; First orders; Step conversion %; Overall visit-to-order %</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Funnel chart with step % drop-off; small-multiples by city/store; trend of overall conversion %</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Quantify drop-off at each step App Visit -&gt; Signup -&gt; Profile Creation -&gt; First Order, sliced by store/city/source to find where we leak demand.. Dependencies: Event instrumentation</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Acquisition Source; Order Channel; City; Store. Granularity: Daily / Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Retention (P0)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>[D03] Retention &amp; RFM</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Cohort retention rate (M0..Mn); Active rate; RFM scores (R,F,M 1-5); RFM segment sizes; repeat rate by segment</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Cohort retention heatmap (triangle); retention curves; RFM 5x5 grid &amp; segment table</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Measure whether acquired customers stick. Cohort retention curves + RFM segmentation, filterable by cohort date range, city, store, acquisition source.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Cohort/date range; City; Store; Acquisition Source; Order Channel; RFM Segment. Granularity: Monthly cohorts (weekly optional)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Acquisition (P0)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>[D04] Order Flow — New vs Repeat</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Total orders; New-customer orders; Repeat-customer orders; New:Repeat ratio; % repeat orders</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Stacked area/bar new vs repeat over time; KPI tiles for D/W/M; ratio trend line</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Track total order volume over time split by new vs repeat, to see if growth is genuine acquisition or just churn-and-replace.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel; Customer Type. Granularity: Daily / Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Monetization (P1)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>[D05] Customer Lifetime Value (CLTV)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Historical CLTV (avg &amp; by segment); Avg orders per customer; Avg revenue per customer; CLTV by RFM segment; CLTV:CAC (if spend joined)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>CFO / Finance Team</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>CLTV distribution; CLTV by source/city/store bars; CLTV:CAC gauge; top-decile customer table</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Understand the value of a customer over their lifetime, by source/city/store, to set sustainable acquisition budgets.. Dependencies: Channel integration; depends on D03</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range (acquisition cohort); Acquisition Source; City; Store; RFM Segment; Order Channel. Granularity: Monthly cohort / lifetime to date</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Retention (P1)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>[D06] Repeat Purchase Gap / Order Velocity</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Median &amp; avg gap 1-&gt;2, 2-&gt;3, 3-&gt;4; % reaching 2nd/3rd/4th order; distribution of inter-order intervals</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Bar of median gap per order-step; survival/repeat-progression funnel; distribution histogram</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Measure the average days between consecutive orders (1st-&gt;2nd, 2nd-&gt;3rd, 3rd-&gt;4th) to time win-back nudges and detect slowing velocity.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel. Granularity: Per order-pair; trended monthly</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Retention (P1)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>[D07] Customer Lifecycle Stage</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Count &amp; % of base per stage: Lead, New, Active, Repeat/Loyal, At-risk, Dormant, Reactivated; stage migration over time</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Funnel/pyramid of stage counts; stage-share trend; migration (sankey/flow) optional</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>A clean single view of how many customers sit in each lifecycle stage so we can see the health of the base at a glance.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date snapshot; City; Store; Acquisition Source; Order Channel. Granularity: Monthly snapshot + migration trend</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Monetization (P0)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>[D08] Revenue</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Total revenue; New vs Repeat revenue; AOV; Revenue per active customer; revenue by source/city/store; MoM/ YoY growth</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>CFO / Finance Team</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Revenue trend with new/repeat stack; KPI tiles; source/city/store contribution bars; growth % line</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Total revenue with new vs repeat split and full filtering, the core money view for leadership and investors.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Acquisition Source; Order Channel; City; Store; Customer Type; Garment/Item Category. Granularity: Daily / Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Efficiency (P0)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>[D09] Marketing Efficiency — CAC, ROAS &amp; Spend</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Spend (Meta/Google/total); Blended &amp; channel CAC; ROAS; CLTV:CAC; CAC payback (months); cost per install; cost per first order</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Data Platform / Tech Team</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>CAC &amp; ROAS trend; spend vs new-customers dual axis; CAC by channel bars; payback gauge</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Connect ad spend to acquired customers &amp; revenue. The single most important view for judging if marketing is efficient and fundraise-ready.. Dependencies: Ads API access; attribution model agreed</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Acquisition Source/Platform; Campaign; City; Store. Granularity: Daily / Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Efficiency (P1)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>[D10] Cohort Revenue &amp; Payback</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Cohort cumulative revenue (M0..Mn); cohort size; revenue per customer over time; months-to-payback; LTV curve</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Data Platform / Tech Team</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Cohort cumulative-revenue triangle; payback line crossing CAC; LTV-by-cohort curves</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Show cumulative revenue per acquisition cohort vs the CAC spent to acquire it — proves unit economics to investors.. Dependencies: Channel integration; depends on D09</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Cohort month; Acquisition Source; City; Store. Granularity: Monthly cohorts</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Store &amp; Geo (P0)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>[D11] Store Performance Scorecard</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Per store: orders, revenue, new vs repeat, AOV, retention rate, CAC, SV customers vs 500 target, MoM growth; red/amber/green flags</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Store Manager / Ops Head</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Sortable scorecard table with RAG conditional formatting; store ranking; map heat by performance</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>One row per store (all 19) scoring orders, revenue, new/repeat, retention, CAC and progress to the 500 SV-customer target — for operational accountability.. Dependencies: Channel integration; ties to SV plan</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel. Granularity: Monthly (with D/W drill)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Store &amp; Geo (P0)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>[D12] Super Value (SV) Customer Tracker</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>SV customers per store; SV vs 500 target &amp; % complete; net new SV per month; SV by source; SV run-rate vs plan</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Store Manager / Ops Head</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Progress bars per store vs 500; actual-vs-plan line; net-new SV trend</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Track progress toward 500 SV customers per store (the core 12-month growth KPI), so the SV acquisition plan is measurable in real time.. Dependencies: Confirm SV definition; channel integration</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel. Granularity: Monthly vs plan</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Foundation (P0)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>[D13] Channel &amp; Attribution Source-of-Truth</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Orders &amp; revenue by channel; channel mix %; % orders missing source; reconciliation vs finance; data-freshness lag</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Data Platform / Tech Team</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Channel-mix donut; orders-by-channel trend; reconciliation table; data-gap flags</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>A unified, reconciled view of every order by Order Channel (App/WhatsApp/Call) with data-completeness QA — the trust layer under all other dashboards.. Dependencies: Channel integration (this dashboard verifies the fix)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Order Channel; City; Store; Acquisition Source. Granularity: Daily</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Retention (P1)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>[D14] Churn &amp; Win-back / Reactivation</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Churn rate; at-risk count; dormant count; reactivation rate; revenue recovered; win-back campaign ROI</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Churn trend; at-risk/dormant counts; reactivation funnel; recovered-revenue tile</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Quantify churn, surface at-risk &amp; dormant customers, and measure whether win-back campaigns actually bring them back.. Dependencies: Channel integration; depends on D07</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel; Lifecycle Stage. Granularity: Monthly</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Conversion (P1)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>[D15] WhatsApp Funnel</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>CTWA clicks; conversations started; qualified leads; orders; step conversion %; cost per WA order</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp funnel chart; cost-per-stage; conversation-to-order %</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Track the Click-to-WhatsApp journey: ad click -&gt; conversation started -&gt; qualified -&gt; order placed, to activate the WhatsApp funnel properly.. Dependencies: Channel integration (WhatsApp) — currently blocked</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Campaign; City; Store. Granularity: Daily / Weekly</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Efficiency (P1)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>[D16] Campaign &amp; Promo / Offer Performance</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Orders/revenue with vs without offer; redemption rate; discount value; incremental orders; new vs repeat on offer; campaign-level ROI</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Data Platform / Tech Team</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Campaign table with ROI; redemption funnel; discount-vs-incremental-revenue chart</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Measure how coupons, offers and campaigns drive orders and whether discounting is incremental or just margin give-away.. Dependencies: Coupon field instrumented</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Campaign/Offer; Acquisition Source; Order Channel; City; Store; Customer Type. Granularity: Per campaign + monthly</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Monetization (P2)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>[D17] AOV &amp; Basket / Item Mix</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>AOV; items per order; revenue/ orders by garment category; category attach rate; AOV trend</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>CFO / Finance Team</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Category contribution bars; items-per-order trend; AOV by category; basket affinity table</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Understand basket composition — which garment categories drive value — to guide pricing, bundles and upsell.. Dependencies: Line-item capture</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Garment/Item Category; City; Store; Order Channel; Customer Type. Granularity: Monthly</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Store &amp; Geo (P2)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>[D18] City / Geo Expansion</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Customers/orders/revenue per city; new-customer density; store coverage; growth by city; CAC by city</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Store Manager / Ops Head</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Geo map heat; city ranking; city growth small-multiples</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>City-level penetration &amp; opportunity view to guide where to expand stores and concentrate marketing.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Acquisition Source; Order Channel. Granularity: Monthly</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Executive (P0)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>[D19] Executive Marketing MIS (North-Star)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>New customers; CAC; CLTV:CAC; repeat rate; revenue &amp; growth; ROAS; SV progress; retention — all vs target &amp; prior period</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Founder &amp; Management</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>KPI tile grid with trend sparklines &amp; RAG vs target; one-page export</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>A single one-screen leadership/investor view of north-star marketing metrics with trend &amp; vs-target — the weekly/monthly decision cockpit.. Dependencies: Depends on D01-D13</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel. Granularity: Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Portal Backend APIs</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>Requires Portal API &amp; UI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Foundation (P0)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>[D20] Data Health &amp; Instrumentation QA</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Event coverage %; channel coverage (App/WA/Call); % orders missing source/store; data freshness/lag; row-count anomalies</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Data Platform / Tech Team</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Coverage scorecard; missing-field heatmap; freshness monitor; anomaly alerts</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Monitor the health of the data feeding every dashboard — event/channel coverage, missing fields, freshness — so we trust the numbers.. Dependencies: Sits on top of channel integration</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Order Channel; Source system. Granularity: Daily / real-time</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000D7377"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>STEAMEE — Metabase + MoEngage (Marketing Architecture)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Dashboard Element Type</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Element Name / Attributes</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>What it Shows (Plain English)</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>Target Portal Role / User</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>Suggested Visualization</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>Business Purpose &amp; Decision Impact</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>Available Filters</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>Source KPI Map</t>
+        </is>
+      </c>
+      <c r="I2" s="13" t="inlineStr">
+        <is>
+          <t>Build Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Acquisition (P0)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>[D01] User Acquisition</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>New customers; New customer orders; AOV (first order); First-order item mix; Spend-to-new ratio (if spend joined)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Trend line of new customers; stacked bar by source; map/table by city &amp; store; item-mix bar; first-order AOV KPI</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>See where new customers come from and what they buy on first order, so we can judge which sources/cities/stores produce quality acquisition.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Acquisition Source; Order Channel; City; Store; Garment/Item Category. Granularity: Daily / Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Conversion (P0)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[D02] User Conversion Funnel</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Visitors; Signups; Profiles created; First orders; Step conversion %; Overall visit-to-order %</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Funnel chart with step % drop-off; small-multiples by city/store; trend of overall conversion %</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Quantify drop-off at each step App Visit -&gt; Signup -&gt; Profile Creation -&gt; First Order, sliced by store/city/source to find where we leak demand.. Dependencies: Event instrumentation</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Acquisition Source; Order Channel; City; Store. Granularity: Daily / Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Retention (P0)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>[D03] Retention &amp; RFM</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Cohort retention rate (M0..Mn); Active rate; RFM scores (R,F,M 1-5); RFM segment sizes; repeat rate by segment</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Cohort retention heatmap (triangle); retention curves; RFM 5x5 grid &amp; segment table</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Measure whether acquired customers stick. Cohort retention curves + RFM segmentation, filterable by cohort date range, city, store, acquisition source.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Cohort/date range; City; Store; Acquisition Source; Order Channel; RFM Segment. Granularity: Monthly cohorts (weekly optional)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Acquisition (P0)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>[D04] Order Flow — New vs Repeat</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Total orders; New-customer orders; Repeat-customer orders; New:Repeat ratio; % repeat orders</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Stacked area/bar new vs repeat over time; KPI tiles for D/W/M; ratio trend line</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Track total order volume over time split by new vs repeat, to see if growth is genuine acquisition or just churn-and-replace.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel; Customer Type. Granularity: Daily / Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Monetization (P1)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>[D05] Customer Lifetime Value (CLTV)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Historical CLTV (avg &amp; by segment); Avg orders per customer; Avg revenue per customer; CLTV by RFM segment; CLTV:CAC (if spend joined)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>CFO / Finance Team</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>CLTV distribution; CLTV by source/city/store bars; CLTV:CAC gauge; top-decile customer table</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Understand the value of a customer over their lifetime, by source/city/store, to set sustainable acquisition budgets.. Dependencies: Channel integration; depends on D03</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range (acquisition cohort); Acquisition Source; City; Store; RFM Segment; Order Channel. Granularity: Monthly cohort / lifetime to date</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Retention (P1)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>[D06] Repeat Purchase Gap / Order Velocity</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Median &amp; avg gap 1-&gt;2, 2-&gt;3, 3-&gt;4; % reaching 2nd/3rd/4th order; distribution of inter-order intervals</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Bar of median gap per order-step; survival/repeat-progression funnel; distribution histogram</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Measure the average days between consecutive orders (1st-&gt;2nd, 2nd-&gt;3rd, 3rd-&gt;4th) to time win-back nudges and detect slowing velocity.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel. Granularity: Per order-pair; trended monthly</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Retention (P1)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>[D07] Customer Lifecycle Stage</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Count &amp; % of base per stage: Lead, New, Active, Repeat/Loyal, At-risk, Dormant, Reactivated; stage migration over time</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Funnel/pyramid of stage counts; stage-share trend; migration (sankey/flow) optional</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>A clean single view of how many customers sit in each lifecycle stage so we can see the health of the base at a glance.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date snapshot; City; Store; Acquisition Source; Order Channel. Granularity: Monthly snapshot + migration trend</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Monetization (P0)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>[D08] Revenue</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Total revenue; New vs Repeat revenue; AOV; Revenue per active customer; revenue by source/city/store; MoM/ YoY growth</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>CFO / Finance Team</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Revenue trend with new/repeat stack; KPI tiles; source/city/store contribution bars; growth % line</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Total revenue with new vs repeat split and full filtering, the core money view for leadership and investors.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Acquisition Source; Order Channel; City; Store; Customer Type; Garment/Item Category. Granularity: Daily / Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Efficiency (P0)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>[D09] Marketing Efficiency — CAC, ROAS &amp; Spend</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Spend (Meta/Google/total); Blended &amp; channel CAC; ROAS; CLTV:CAC; CAC payback (months); cost per install; cost per first order</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Data Platform / Tech Team</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>CAC &amp; ROAS trend; spend vs new-customers dual axis; CAC by channel bars; payback gauge</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Connect ad spend to acquired customers &amp; revenue. The single most important view for judging if marketing is efficient and fundraise-ready.. Dependencies: Ads API access; attribution model agreed</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Acquisition Source/Platform; Campaign; City; Store. Granularity: Daily / Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Efficiency (P1)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>[D10] Cohort Revenue &amp; Payback</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Cohort cumulative revenue (M0..Mn); cohort size; revenue per customer over time; months-to-payback; LTV curve</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Data Platform / Tech Team</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Cohort cumulative-revenue triangle; payback line crossing CAC; LTV-by-cohort curves</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Show cumulative revenue per acquisition cohort vs the CAC spent to acquire it — proves unit economics to investors.. Dependencies: Channel integration; depends on D09</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Cohort month; Acquisition Source; City; Store. Granularity: Monthly cohorts</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Store &amp; Geo (P0)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>[D11] Store Performance Scorecard</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Per store: orders, revenue, new vs repeat, AOV, retention rate, CAC, SV customers vs 500 target, MoM growth; red/amber/green flags</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Store Manager / Ops Head</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Sortable scorecard table with RAG conditional formatting; store ranking; map heat by performance</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>One row per store (all 19) scoring orders, revenue, new/repeat, retention, CAC and progress to the 500 SV-customer target — for operational accountability.. Dependencies: Channel integration; ties to SV plan</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel. Granularity: Monthly (with D/W drill)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Store &amp; Geo (P0)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>[D12] Super Value (SV) Customer Tracker</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>SV customers per store; SV vs 500 target &amp; % complete; net new SV per month; SV by source; SV run-rate vs plan</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Store Manager / Ops Head</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Progress bars per store vs 500; actual-vs-plan line; net-new SV trend</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Track progress toward 500 SV customers per store (the core 12-month growth KPI), so the SV acquisition plan is measurable in real time.. Dependencies: Confirm SV definition; channel integration</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel. Granularity: Monthly vs plan</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Foundation (P0)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>[D13] Channel &amp; Attribution Source-of-Truth</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Orders &amp; revenue by channel; channel mix %; % orders missing source; reconciliation vs finance; data-freshness lag</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Data Platform / Tech Team</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Channel-mix donut; orders-by-channel trend; reconciliation table; data-gap flags</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>A unified, reconciled view of every order by Order Channel (App/WhatsApp/Call) with data-completeness QA — the trust layer under all other dashboards.. Dependencies: Channel integration (this dashboard verifies the fix)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Order Channel; City; Store; Acquisition Source. Granularity: Daily</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Retention (P1)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>[D14] Churn &amp; Win-back / Reactivation</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Churn rate; at-risk count; dormant count; reactivation rate; revenue recovered; win-back campaign ROI</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Churn trend; at-risk/dormant counts; reactivation funnel; recovered-revenue tile</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Quantify churn, surface at-risk &amp; dormant customers, and measure whether win-back campaigns actually bring them back.. Dependencies: Channel integration; depends on D07</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel; Lifecycle Stage. Granularity: Monthly</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Conversion (P1)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>[D15] WhatsApp Funnel</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>CTWA clicks; conversations started; qualified leads; orders; step conversion %; cost per WA order</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Growth Team</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp funnel chart; cost-per-stage; conversation-to-order %</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Track the Click-to-WhatsApp journey: ad click -&gt; conversation started -&gt; qualified -&gt; order placed, to activate the WhatsApp funnel properly.. Dependencies: Channel integration (WhatsApp) — currently blocked</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Campaign; City; Store. Granularity: Daily / Weekly</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Efficiency (P1)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>[D16] Campaign &amp; Promo / Offer Performance</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Orders/revenue with vs without offer; redemption rate; discount value; incremental orders; new vs repeat on offer; campaign-level ROI</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Data Platform / Tech Team</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Campaign table with ROI; redemption funnel; discount-vs-incremental-revenue chart</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Measure how coupons, offers and campaigns drive orders and whether discounting is incremental or just margin give-away.. Dependencies: Coupon field instrumented</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Campaign/Offer; Acquisition Source; Order Channel; City; Store; Customer Type. Granularity: Per campaign + monthly</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Monetization (P2)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>[D17] AOV &amp; Basket / Item Mix</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>AOV; items per order; revenue/ orders by garment category; category attach rate; AOV trend</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>CFO / Finance Team</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Category contribution bars; items-per-order trend; AOV by category; basket affinity table</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Understand basket composition — which garment categories drive value — to guide pricing, bundles and upsell.. Dependencies: Line-item capture</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Garment/Item Category; City; Store; Order Channel; Customer Type. Granularity: Monthly</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Store &amp; Geo (P2)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>[D18] City / Geo Expansion</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Customers/orders/revenue per city; new-customer density; store coverage; growth by city; CAC by city</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Store Manager / Ops Head</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Geo map heat; city ranking; city growth small-multiples</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>City-level penetration &amp; opportunity view to guide where to expand stores and concentrate marketing.. Dependencies: Channel integration</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Acquisition Source; Order Channel. Granularity: Monthly</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Executive (P0)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>[D19] Executive Marketing MIS (North-Star)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>New customers; CAC; CLTV:CAC; repeat rate; revenue &amp; growth; ROAS; SV progress; retention — all vs target &amp; prior period</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Founder &amp; Management</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>KPI tile grid with trend sparklines &amp; RAG vs target; one-page export</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>A single one-screen leadership/investor view of north-star marketing metrics with trend &amp; vs-target — the weekly/monthly decision cockpit.. Dependencies: Depends on D01-D13</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; City; Store; Acquisition Source; Order Channel. Granularity: Weekly / Monthly</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Metabase SQL / Postgres</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (SQL Metabase Query)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Foundation (P0)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>[D20] Data Health &amp; Instrumentation QA</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Event coverage %; channel coverage (App/WA/Call); % orders missing source/store; data freshness/lag; row-count anomalies</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Data Platform / Tech Team</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Coverage scorecard; missing-field heatmap; freshness monitor; anomaly alerts</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Monitor the health of the data feeding every dashboard — event/channel coverage, missing fields, freshness — so we trust the numbers.. Dependencies: Sits on top of channel integration</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions: Date range; Order Channel; Source system. Granularity: Daily / real-time</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>MoEngage Events</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Ready to Build (MoEngage Event)</t>
         </is>
       </c>
     </row>
@@ -3200,7 +5268,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -4693,7 +6761,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -5998,7 +8066,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -6645,7 +8713,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -7997,7 +10065,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -8550,7 +10618,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -9150,7 +11218,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -9750,7 +11818,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>

</xml_diff>